<commit_message>
Arrancar el assessment sin puntuaciones de ejemplo
La subcapacidad 1.1 de FP&A venia puntuada 2/4/3 desde el Excel, herencia
de la fila de ejemplo con la que se monto la plantilla. La herramienta
abria mostrando "Score global 3" y "1/20, 5% de avance" sin que nadie
hubiera evaluado nada, y era la primera cifra que veia un cliente en una
sesion de arranque. Es la unica de las 152 subcapacidades que lo hacia.

Se vacian las tres celdas en el Excel de origen y se regenera fpa.json.

La edicion se hace sobre el XML de la hoja y no con openpyxl: el libro
lleva un grafico en la hoja Resumen que openpyxl no sabe conservar al
guardar. Se tocan solo I2, J2 y K2; las formulas de las columnas
derivadas se quedan como estan, porque la fila 2 contiene la definicion
maestra de las formulas compartidas de toda la columna. Excel recalcula
esos valores al abrir el archivo.

check_domains_sync.py sigue en verde para los nueve dominios.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/F3M_FP&A_assessment_ready_AI_v1.xlsx
+++ b/F3M_FP&A_assessment_ready_AI_v1.xlsx
@@ -1870,15 +1870,9 @@
       <c r="H2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="1">
-        <v>2</v>
-      </c>
-      <c r="J2" s="1">
-        <v>4</v>
-      </c>
-      <c r="K2" s="1">
-        <v>3</v>
-      </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
       <c r="L2" s="1">
         <f t="shared" ref="L2:L21" si="0">IF(COUNTA(I2:K2)=0,"",ROUND(AVERAGE(I2:K2),2))</f>
         <v>3</v>

</xml_diff>